<commit_message>
id19bom STYD40000608-4021 BOM明細表示 fix: fetchBOMItems をAPIフィルタに任せ、/bom-items/?bom=ID のレスポンスをそのまま表示
</commit_message>
<xml_diff>
--- a/bom_tree (シミュレーション).xlsx
+++ b/bom_tree (シミュレーション).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00C1C63-D3A5-4CD6-8F1C-ED4EFADCC0ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A10F8A-CF09-442A-95E9-13FC43014DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Tree" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="109">
   <si>
     <t>BOM ID</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>4007 - タンク小組</t>
-  </si>
-  <si>
-    <t>L2202 - タンク艤装</t>
   </si>
   <si>
     <t>├─ YD60000441S</t>
@@ -351,10 +348,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>L2202 - タンク艤装</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>サイクル時間</t>
     <rPh sb="4" eb="6">
       <t>ジカン</t>
@@ -371,6 +364,9 @@
   <si>
     <t>リードタイム</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>L2200 - タンクライン</t>
   </si>
 </sst>
 </file>
@@ -717,7 +713,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K59"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
@@ -756,16 +751,16 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J1" t="s">
+        <v>105</v>
+      </c>
+      <c r="K1" t="s">
         <v>107</v>
       </c>
-      <c r="K1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -782,16 +777,16 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J2">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -799,36 +794,36 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
       <c r="G3" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J3">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -837,13 +832,13 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J4">
         <v>19</v>
@@ -854,10 +849,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -866,27 +861,27 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
         <v>19</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
+        <v>106</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>108</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -895,42 +890,42 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J6">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
         <v>24</v>
       </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>25</v>
-      </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J7">
         <v>15</v>
@@ -941,22 +936,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
         <v>27</v>
       </c>
-      <c r="D8">
-        <v>5</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="H8" t="s">
-        <v>28</v>
-      </c>
       <c r="I8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K8">
         <v>3</v>
@@ -967,10 +962,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D9">
         <v>5</v>
@@ -979,24 +974,24 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K9">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -1005,13 +1000,13 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J10">
         <v>15</v>
@@ -1022,69 +1017,69 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
         <v>31</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" t="s">
+        <v>106</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
         <v>32</v>
       </c>
-      <c r="D11">
-        <v>5</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" t="s">
         <v>108</v>
       </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" t="s">
-        <v>11</v>
-      </c>
       <c r="I12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J12">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>7</v>
       </c>
       <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="C13" t="s">
-        <v>35</v>
-      </c>
       <c r="D13">
         <v>5</v>
       </c>
@@ -1092,13 +1087,13 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G13" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J13">
         <v>15</v>
@@ -1109,10 +1104,10 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" t="s">
         <v>36</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
       </c>
       <c r="D14">
         <v>6</v>
@@ -1121,13 +1116,13 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
         <v>19</v>
       </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
       <c r="I14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -1138,10 +1133,10 @@
         <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D15">
         <v>5</v>
@@ -1150,10 +1145,10 @@
         <v>2</v>
       </c>
       <c r="H15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K15">
         <v>1</v>
@@ -1164,22 +1159,22 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="H16" t="s">
         <v>40</v>
       </c>
-      <c r="D16">
-        <v>5</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="H16" t="s">
-        <v>41</v>
-      </c>
       <c r="I16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K16">
         <v>30</v>
@@ -1190,22 +1185,22 @@
         <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="H17" t="s">
         <v>42</v>
       </c>
-      <c r="D17">
-        <v>5</v>
-      </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="H17" t="s">
-        <v>43</v>
-      </c>
       <c r="I17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K17">
         <v>1</v>
@@ -1216,22 +1211,22 @@
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
         <v>44</v>
       </c>
-      <c r="D18">
-        <v>5</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="H18" t="s">
-        <v>45</v>
-      </c>
       <c r="I18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -1242,22 +1237,22 @@
         <v>7</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="H19" t="s">
         <v>46</v>
       </c>
-      <c r="D19">
-        <v>5</v>
-      </c>
-      <c r="E19">
-        <v>1</v>
-      </c>
-      <c r="H19" t="s">
-        <v>47</v>
-      </c>
       <c r="I19" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K19">
         <v>1</v>
@@ -1268,22 +1263,22 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="H20" t="s">
         <v>48</v>
       </c>
-      <c r="D20">
-        <v>5</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="H20" t="s">
-        <v>49</v>
-      </c>
       <c r="I20" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -1294,25 +1289,25 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
         <v>50</v>
       </c>
-      <c r="D21">
-        <v>4</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>51</v>
       </c>
-      <c r="G21" t="s">
-        <v>52</v>
-      </c>
       <c r="I21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K21">
         <v>1</v>
@@ -1323,39 +1318,39 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" t="s">
         <v>53</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22">
+        <v>5</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" t="s">
+        <v>19</v>
+      </c>
+      <c r="I22" t="s">
+        <v>106</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
         <v>54</v>
-      </c>
-      <c r="D22">
-        <v>5</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" t="s">
-        <v>20</v>
-      </c>
-      <c r="I22" t="s">
-        <v>108</v>
-      </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" t="s">
-        <v>55</v>
       </c>
       <c r="D23">
         <v>4</v>
@@ -1364,13 +1359,13 @@
         <v>2</v>
       </c>
       <c r="F23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G23" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="I23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J23">
         <v>15</v>
@@ -1381,22 +1376,22 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" t="s">
         <v>56</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24">
+        <v>5</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="H24" t="s">
         <v>57</v>
       </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="H24" t="s">
-        <v>58</v>
-      </c>
       <c r="I24" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K24">
         <v>1</v>
@@ -1407,22 +1402,22 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="H25" t="s">
         <v>59</v>
       </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="H25" t="s">
-        <v>60</v>
-      </c>
       <c r="I25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K25">
         <v>1</v>
@@ -1433,10 +1428,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D26">
         <v>4</v>
@@ -1445,10 +1440,10 @@
         <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K26">
         <v>1</v>
@@ -1459,10 +1454,10 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D27">
         <v>4</v>
@@ -1471,10 +1466,10 @@
         <v>2</v>
       </c>
       <c r="H27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I27" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K27">
         <v>1</v>
@@ -1485,10 +1480,10 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D28">
         <v>3</v>
@@ -1497,13 +1492,13 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" t="s">
         <v>65</v>
       </c>
-      <c r="G28" t="s">
-        <v>66</v>
-      </c>
       <c r="I28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K28">
         <v>1</v>
@@ -1514,22 +1509,22 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" t="s">
         <v>67</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29">
+        <v>4</v>
+      </c>
+      <c r="H29" t="s">
         <v>68</v>
       </c>
-      <c r="D29">
-        <v>4</v>
-      </c>
-      <c r="E29">
-        <v>4</v>
-      </c>
-      <c r="H29" t="s">
-        <v>69</v>
-      </c>
       <c r="I29" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K29">
         <v>1</v>
@@ -1540,10 +1535,10 @@
         <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30">
         <v>4</v>
@@ -1552,10 +1547,10 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I30" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K30">
         <v>1</v>
@@ -1566,10 +1561,10 @@
         <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31">
         <v>3</v>
@@ -1578,10 +1573,10 @@
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K31">
         <v>1</v>
@@ -1592,10 +1587,10 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D32">
         <v>3</v>
@@ -1604,10 +1599,10 @@
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I32" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K32">
         <v>1</v>
@@ -1618,10 +1613,10 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D33">
         <v>3</v>
@@ -1630,10 +1625,10 @@
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I33" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K33">
         <v>1</v>
@@ -1644,10 +1639,10 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D34">
         <v>3</v>
@@ -1656,10 +1651,10 @@
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I34" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K34">
         <v>30</v>
@@ -1670,10 +1665,10 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D35">
         <v>3</v>
@@ -1682,13 +1677,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" t="s">
         <v>51</v>
       </c>
-      <c r="G35" t="s">
-        <v>52</v>
-      </c>
       <c r="I35" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K35">
         <v>1</v>
@@ -1699,11 +1694,11 @@
         <v>13</v>
       </c>
       <c r="B36" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" t="s">
         <v>76</v>
       </c>
-      <c r="C36" t="s">
-        <v>77</v>
-      </c>
       <c r="D36">
         <v>4</v>
       </c>
@@ -1711,13 +1706,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" t="s">
         <v>19</v>
       </c>
-      <c r="G36" t="s">
-        <v>20</v>
-      </c>
       <c r="I36" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K36">
         <v>1</v>
@@ -1728,10 +1723,10 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D37">
         <v>3</v>
@@ -1740,13 +1735,13 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" t="s">
         <v>65</v>
       </c>
-      <c r="G37" t="s">
-        <v>66</v>
-      </c>
       <c r="I37" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K37">
         <v>1</v>
@@ -1757,11 +1752,11 @@
         <v>18</v>
       </c>
       <c r="B38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" t="s">
         <v>79</v>
       </c>
-      <c r="C38" t="s">
-        <v>80</v>
-      </c>
       <c r="D38">
         <v>4</v>
       </c>
@@ -1769,10 +1764,10 @@
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I38" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -1783,10 +1778,10 @@
         <v>18</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -1795,10 +1790,10 @@
         <v>6</v>
       </c>
       <c r="H39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I39" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K39">
         <v>1</v>
@@ -1812,7 +1807,7 @@
         <v>8</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1821,10 +1816,10 @@
         <v>2</v>
       </c>
       <c r="H40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I40" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K40">
         <v>1</v>
@@ -1838,7 +1833,7 @@
         <v>8</v>
       </c>
       <c r="C41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1847,10 +1842,10 @@
         <v>2</v>
       </c>
       <c r="H41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K41">
         <v>1</v>
@@ -1864,7 +1859,7 @@
         <v>8</v>
       </c>
       <c r="C42" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1873,10 +1868,10 @@
         <v>6</v>
       </c>
       <c r="H42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I42" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K42">
         <v>1</v>
@@ -1890,7 +1885,7 @@
         <v>8</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1899,10 +1894,10 @@
         <v>4</v>
       </c>
       <c r="H43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I43" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K43">
         <v>5</v>
@@ -1916,7 +1911,7 @@
         <v>8</v>
       </c>
       <c r="C44" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1925,10 +1920,10 @@
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I44" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K44">
         <v>5</v>
@@ -1942,7 +1937,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1951,10 +1946,10 @@
         <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I45" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K45">
         <v>1</v>
@@ -1968,7 +1963,7 @@
         <v>8</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -1977,10 +1972,10 @@
         <v>2</v>
       </c>
       <c r="H46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I46" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K46">
         <v>2</v>
@@ -1994,7 +1989,7 @@
         <v>8</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -2003,10 +1998,10 @@
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K47">
         <v>2</v>
@@ -2020,7 +2015,7 @@
         <v>8</v>
       </c>
       <c r="C48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -2029,10 +2024,10 @@
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K48">
         <v>2</v>
@@ -2046,7 +2041,7 @@
         <v>8</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -2055,10 +2050,10 @@
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I49" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K49">
         <v>2</v>
@@ -2072,7 +2067,7 @@
         <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -2081,10 +2076,10 @@
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I50" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K50">
         <v>10</v>
@@ -2098,7 +2093,7 @@
         <v>8</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -2107,10 +2102,10 @@
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I51" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K51">
         <v>5</v>
@@ -2124,7 +2119,7 @@
         <v>8</v>
       </c>
       <c r="C52" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -2133,10 +2128,10 @@
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I52" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K52">
         <v>5</v>
@@ -2150,7 +2145,7 @@
         <v>8</v>
       </c>
       <c r="C53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -2159,10 +2154,10 @@
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I53" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K53">
         <v>5</v>
@@ -2176,7 +2171,7 @@
         <v>8</v>
       </c>
       <c r="C54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -2185,10 +2180,10 @@
         <v>1</v>
       </c>
       <c r="H54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I54" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K54">
         <v>5</v>
@@ -2202,7 +2197,7 @@
         <v>8</v>
       </c>
       <c r="C55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -2211,10 +2206,10 @@
         <v>1</v>
       </c>
       <c r="H55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K55">
         <v>5</v>
@@ -2228,7 +2223,7 @@
         <v>8</v>
       </c>
       <c r="C56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -2237,10 +2232,10 @@
         <v>3</v>
       </c>
       <c r="H56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I56" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K56">
         <v>5</v>
@@ -2254,7 +2249,7 @@
         <v>8</v>
       </c>
       <c r="C57" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -2263,10 +2258,10 @@
         <v>2</v>
       </c>
       <c r="H57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I57" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K57">
         <v>5</v>
@@ -2280,7 +2275,7 @@
         <v>8</v>
       </c>
       <c r="C58" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -2289,28 +2284,22 @@
         <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I58" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K58">
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="I59" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I59" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="日"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I59" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
画面を src/views/{masters,orders,production,purchase,shipping}/ に再配置し、旧 src/pages を削除。 vite.config.js に @ エイリアスを追加し、各画面の import を @/api/client / @/utils/dateUtil に更新。 ルーターをドメイン別に分割（src/router/masters.js, orders.js, production.js, purchase.js, shipping.js）。src/router/index.js は各モジュールを結合しつつルート /→/masters を維持。
</commit_message>
<xml_diff>
--- a/bom_tree (シミュレーション).xlsx
+++ b/bom_tree (シミュレーション).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A10F8A-CF09-442A-95E9-13FC43014DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FB3CCD-7266-4F87-BA97-8B07686AA088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Tree" sheetId="1" r:id="rId1"/>
@@ -713,6 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K59"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
@@ -760,7 +761,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -786,7 +787,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -815,7 +816,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -844,7 +845,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -873,7 +874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -931,7 +932,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -957,7 +958,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6</v>
       </c>
@@ -1012,7 +1013,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1099,7 +1100,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>14</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>7</v>
       </c>
@@ -1154,7 +1155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>7</v>
       </c>
@@ -1180,7 +1181,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>7</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>7</v>
       </c>
@@ -1232,7 +1233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>7</v>
       </c>
@@ -1258,7 +1259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>7</v>
       </c>
@@ -1284,7 +1285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>5</v>
       </c>
@@ -1313,7 +1314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>16</v>
       </c>
@@ -1371,7 +1372,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>8</v>
       </c>
@@ -1397,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>8</v>
       </c>
@@ -1423,7 +1424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>5</v>
       </c>
@@ -1449,7 +1450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>5</v>
       </c>
@@ -1475,7 +1476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1504,7 +1505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>17</v>
       </c>
@@ -1530,7 +1531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>17</v>
       </c>
@@ -1556,7 +1557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1582,7 +1583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1608,7 +1609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1634,7 +1635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4</v>
       </c>
@@ -1660,7 +1661,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4</v>
       </c>
@@ -1689,7 +1690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>13</v>
       </c>
@@ -1718,7 +1719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4</v>
       </c>
@@ -1747,7 +1748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>18</v>
       </c>
@@ -1773,7 +1774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>18</v>
       </c>
@@ -1799,7 +1800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1</v>
       </c>
@@ -1825,7 +1826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1</v>
       </c>
@@ -1851,7 +1852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1</v>
       </c>
@@ -1877,7 +1878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
@@ -1903,7 +1904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1</v>
       </c>
@@ -1929,7 +1930,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1</v>
       </c>
@@ -1955,7 +1956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>1</v>
       </c>
@@ -1981,7 +1982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1</v>
       </c>
@@ -2007,7 +2008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>1</v>
       </c>
@@ -2033,7 +2034,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1</v>
       </c>
@@ -2059,7 +2060,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1</v>
       </c>
@@ -2085,7 +2086,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>1</v>
       </c>
@@ -2111,7 +2112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1</v>
       </c>
@@ -2137,7 +2138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>1</v>
       </c>
@@ -2163,7 +2164,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>1</v>
       </c>
@@ -2189,7 +2190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>1</v>
       </c>
@@ -2215,7 +2216,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>1</v>
       </c>
@@ -2241,7 +2242,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>1</v>
       </c>
@@ -2267,7 +2268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>1</v>
       </c>
@@ -2293,13 +2294,19 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="I59" t="s">
         <v>104</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I59" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I59" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="4021 - タンクサブ―"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>